<commit_message>
Report fitted feature weights for the chosen model
Ridge coefficients (or XGBoost gain importance) are printed by the final
forecast and by backtest.py, and exported to model_weights.csv and a
model_weights sheet in the Excel outputs.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SzFCGFJh2C1KowwkbV591B
</commit_message>
<xml_diff>
--- a/output/backtest_Dec-24.xlsx
+++ b/output/backtest_Dec-24.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet name="stocks" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="model_scores" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="model_weights" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -72168,4 +72169,80 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>feature</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>weight_%</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>size_rank_pct</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>-19.42310484116329</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>intercept</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>11.69197691356176</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>share_chg_1_pct</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>-7.902604814388899</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>rel_return_1_pct</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>-7.413513704065751</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>size_rank_chg_pct</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>0.2004529317868716</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>